<commit_message>
Zusatzanalysen: Dimensionseffekte einzeln und Per-Thema-Embedding mit Fisher-Z
- analysis.py: Zusatzanalyse je einzelner Dimension (between-subjects, N=161,
  Holm-Bonferroni über 10 Tests) -> Dimension_Effekte.xlsx, Plot 12.
  Keine der Korrelationen signifikant
- wordembedding_pertopic.py (neu, eigenständige Pipeline): Prompts pro Thema
  einzeln einbetten, themenspezifische Profilkorrelationen per Fisher-Z
  mitteln. Bestehende aggregierte Pipeline bleibt unverändert daneben
  bestehen. Mean r = +0.004 vs. -0.010 aggregiert -> Aggregation erklärt den
  Nullbefund nicht. Liest Rohdaten.xlsx (liegt nicht im Repo)
- Ergebnis-Dateien und Vergleichsplot 11 neu generiert

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Embedding_Analysis.xlsx
+++ b/Embedding_Analysis.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>